<commit_message>
Birim ve görünen ad rapor-duzeni.xlsx'ten yönetilsin
Kullanıcı bazı ürünlerde "(adet)" ekini kaldırmak ve bazılarının adını
raporda değiştirmek istedi. İkisi de artık düzen dosyasından yapılıyor,
kod değişikliği gerekmiyor:

- birim sütunu yetkili: doluysa parantezde o yazılır, BOŞ bırakılırsa
  ürünün yanında hiç birim yazılmaz (önceden kaydın kendi birimi
  yazılıyordu ve dosyadaki sütun sadece bilgi amaçlıydı).
- Yeni "GÖRÜNEN AD" sütunu: raporda bu ad basılır, boşsa ÜRÜN sütunundaki
  ad kullanılır. ÜRÜN sütunu sistemin anahtarı olduğu için değişmeden
  kalıyor; böylece geçmiş kayıtlarla bağ kopmuyor.

raporAdi() ikisini birleştiriyor ve "(Boy 2)" gibi ekleri koruyor
(ör. "Ganaj (Klasik) (Boy 2)" -> "Ganaj Boylu (Boy 2)"). Excel ve
panelden yazdırma çıktılarının tamamında aynı fonksiyon kullanılıyor.

Aciklama sayfasındaki yönergeler de güncellendi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,9 @@
       <family val="2"/>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -112,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -127,6 +130,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G224"/>
+  <dimension ref="A1:H224"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -502,6 +506,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -540,6 +545,11 @@
           <t>ALT GRUP</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>GÖRÜNEN AD</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -567,6 +577,7 @@
       </c>
       <c r="F2" s="5" t="n"/>
       <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -592,6 +603,7 @@
       </c>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -619,6 +631,7 @@
       </c>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -646,6 +659,7 @@
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -673,6 +687,7 @@
       </c>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -700,6 +715,7 @@
       </c>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -727,6 +743,7 @@
       </c>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -754,6 +771,7 @@
       </c>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -781,6 +799,7 @@
       </c>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -808,6 +827,7 @@
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -835,6 +855,7 @@
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -862,6 +883,7 @@
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -889,6 +911,7 @@
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -916,6 +939,7 @@
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -943,6 +967,7 @@
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -970,6 +995,7 @@
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -997,6 +1023,7 @@
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1024,6 +1051,7 @@
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1051,6 +1079,7 @@
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1078,6 +1107,7 @@
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1105,6 +1135,7 @@
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1132,6 +1163,7 @@
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1159,6 +1191,7 @@
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1186,6 +1219,7 @@
       </c>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1213,6 +1247,7 @@
       </c>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1244,6 +1279,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1275,6 +1311,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1306,6 +1343,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1337,6 +1375,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1368,6 +1407,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1399,6 +1439,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1430,6 +1471,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1457,6 +1499,7 @@
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1484,6 +1527,7 @@
       </c>
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1511,6 +1555,7 @@
       </c>
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1538,6 +1583,7 @@
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1565,6 +1611,7 @@
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="9" t="n"/>
+      <c r="H38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1592,6 +1639,7 @@
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -1619,6 +1667,7 @@
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1650,6 +1699,7 @@
         </is>
       </c>
       <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -1681,6 +1731,7 @@
         </is>
       </c>
       <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -1712,6 +1763,7 @@
         </is>
       </c>
       <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -1743,6 +1795,7 @@
         </is>
       </c>
       <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1774,6 +1827,7 @@
         </is>
       </c>
       <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -1805,6 +1859,7 @@
         </is>
       </c>
       <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -1836,6 +1891,7 @@
         </is>
       </c>
       <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1867,6 +1923,7 @@
         </is>
       </c>
       <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1898,6 +1955,7 @@
         </is>
       </c>
       <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -1929,6 +1987,7 @@
         </is>
       </c>
       <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1960,6 +2019,7 @@
         </is>
       </c>
       <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -1991,6 +2051,7 @@
         </is>
       </c>
       <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2022,6 +2083,7 @@
         </is>
       </c>
       <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -2053,6 +2115,7 @@
         </is>
       </c>
       <c r="G54" s="9" t="n"/>
+      <c r="H54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2084,6 +2147,7 @@
         </is>
       </c>
       <c r="G55" s="9" t="n"/>
+      <c r="H55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -2115,6 +2179,7 @@
         </is>
       </c>
       <c r="G56" s="9" t="n"/>
+      <c r="H56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2146,6 +2211,7 @@
         </is>
       </c>
       <c r="G57" s="9" t="n"/>
+      <c r="H57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -2177,6 +2243,7 @@
         </is>
       </c>
       <c r="G58" s="9" t="n"/>
+      <c r="H58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2208,6 +2275,7 @@
         </is>
       </c>
       <c r="G59" s="9" t="n"/>
+      <c r="H59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2239,6 +2307,7 @@
         </is>
       </c>
       <c r="G60" s="9" t="n"/>
+      <c r="H60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2270,6 +2339,7 @@
         </is>
       </c>
       <c r="G61" s="9" t="n"/>
+      <c r="H61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2301,6 +2371,7 @@
         </is>
       </c>
       <c r="G62" s="9" t="n"/>
+      <c r="H62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2332,6 +2403,7 @@
         </is>
       </c>
       <c r="G63" s="9" t="n"/>
+      <c r="H63" s="9" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -2363,6 +2435,7 @@
         </is>
       </c>
       <c r="G64" s="9" t="n"/>
+      <c r="H64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2394,6 +2467,7 @@
         </is>
       </c>
       <c r="G65" s="9" t="n"/>
+      <c r="H65" s="9" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -2425,6 +2499,7 @@
         </is>
       </c>
       <c r="G66" s="9" t="n"/>
+      <c r="H66" s="9" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -2456,6 +2531,7 @@
         </is>
       </c>
       <c r="G67" s="9" t="n"/>
+      <c r="H67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -2487,6 +2563,7 @@
         </is>
       </c>
       <c r="G68" s="9" t="n"/>
+      <c r="H68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -2518,6 +2595,7 @@
         </is>
       </c>
       <c r="G69" s="9" t="n"/>
+      <c r="H69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -2549,6 +2627,7 @@
         </is>
       </c>
       <c r="G70" s="9" t="n"/>
+      <c r="H70" s="9" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -2576,6 +2655,7 @@
       </c>
       <c r="F71" s="5" t="n"/>
       <c r="G71" s="9" t="n"/>
+      <c r="H71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -2603,6 +2683,7 @@
       </c>
       <c r="F72" s="5" t="n"/>
       <c r="G72" s="9" t="n"/>
+      <c r="H72" s="9" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2634,6 +2715,7 @@
           <t>Coco</t>
         </is>
       </c>
+      <c r="H73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -2665,6 +2747,7 @@
           <t>Coco</t>
         </is>
       </c>
+      <c r="H74" s="9" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -2696,6 +2779,7 @@
           <t>Coco</t>
         </is>
       </c>
+      <c r="H75" s="9" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -2723,6 +2807,7 @@
       </c>
       <c r="F76" s="5" t="n"/>
       <c r="G76" s="9" t="n"/>
+      <c r="H76" s="9" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -2750,6 +2835,7 @@
       </c>
       <c r="F77" s="5" t="n"/>
       <c r="G77" s="9" t="n"/>
+      <c r="H77" s="9" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -2781,6 +2867,7 @@
           <t>Mekik</t>
         </is>
       </c>
+      <c r="H78" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -2812,6 +2899,7 @@
           <t>Mekik</t>
         </is>
       </c>
+      <c r="H79" s="9" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -2843,6 +2931,7 @@
           <t>Mekik</t>
         </is>
       </c>
+      <c r="H80" s="9" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -2870,6 +2959,7 @@
       </c>
       <c r="F81" s="5" t="n"/>
       <c r="G81" s="9" t="n"/>
+      <c r="H81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -2897,6 +2987,7 @@
       </c>
       <c r="F82" s="5" t="n"/>
       <c r="G82" s="9" t="n"/>
+      <c r="H82" s="9" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -2924,6 +3015,7 @@
       </c>
       <c r="F83" s="5" t="n"/>
       <c r="G83" s="9" t="n"/>
+      <c r="H83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -2951,6 +3043,7 @@
       </c>
       <c r="F84" s="5" t="n"/>
       <c r="G84" s="9" t="n"/>
+      <c r="H84" s="9" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -2978,6 +3071,7 @@
       </c>
       <c r="F85" s="5" t="n"/>
       <c r="G85" s="9" t="n"/>
+      <c r="H85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -3005,6 +3099,7 @@
       </c>
       <c r="F86" s="5" t="n"/>
       <c r="G86" s="9" t="n"/>
+      <c r="H86" s="9" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -3032,6 +3127,7 @@
       </c>
       <c r="F87" s="5" t="n"/>
       <c r="G87" s="9" t="n"/>
+      <c r="H87" s="9" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -3059,6 +3155,7 @@
       </c>
       <c r="F88" s="5" t="n"/>
       <c r="G88" s="9" t="n"/>
+      <c r="H88" s="9" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -3090,6 +3187,7 @@
           <t>Top</t>
         </is>
       </c>
+      <c r="H89" s="9" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -3121,6 +3219,7 @@
           <t>Top</t>
         </is>
       </c>
+      <c r="H90" s="9" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -3152,6 +3251,7 @@
           <t>Top</t>
         </is>
       </c>
+      <c r="H91" s="9" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -3179,6 +3279,7 @@
       </c>
       <c r="F92" s="5" t="n"/>
       <c r="G92" s="9" t="n"/>
+      <c r="H92" s="9" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -3206,6 +3307,7 @@
       </c>
       <c r="F93" s="5" t="n"/>
       <c r="G93" s="9" t="n"/>
+      <c r="H93" s="9" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -3233,6 +3335,7 @@
       </c>
       <c r="F94" s="5" t="n"/>
       <c r="G94" s="9" t="n"/>
+      <c r="H94" s="9" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -3264,6 +3367,7 @@
           <t>Bar</t>
         </is>
       </c>
+      <c r="H95" s="9" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -3295,6 +3399,7 @@
           <t>Bar</t>
         </is>
       </c>
+      <c r="H96" s="9" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -3326,6 +3431,7 @@
           <t>Bar</t>
         </is>
       </c>
+      <c r="H97" s="9" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -3353,6 +3459,7 @@
       </c>
       <c r="F98" s="5" t="n"/>
       <c r="G98" s="9" t="n"/>
+      <c r="H98" s="9" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -3380,6 +3487,7 @@
       </c>
       <c r="F99" s="5" t="n"/>
       <c r="G99" s="9" t="n"/>
+      <c r="H99" s="9" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -3407,6 +3515,7 @@
       </c>
       <c r="F100" s="5" t="n"/>
       <c r="G100" s="9" t="n"/>
+      <c r="H100" s="9" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -3434,6 +3543,7 @@
       </c>
       <c r="F101" s="5" t="n"/>
       <c r="G101" s="9" t="n"/>
+      <c r="H101" s="9" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -3461,6 +3571,7 @@
       </c>
       <c r="F102" s="5" t="n"/>
       <c r="G102" s="9" t="n"/>
+      <c r="H102" s="9" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -3488,6 +3599,7 @@
       </c>
       <c r="F103" s="5" t="n"/>
       <c r="G103" s="9" t="n"/>
+      <c r="H103" s="9" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -3515,6 +3627,7 @@
       </c>
       <c r="F104" s="5" t="n"/>
       <c r="G104" s="9" t="n"/>
+      <c r="H104" s="9" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -3542,6 +3655,7 @@
       </c>
       <c r="F105" s="5" t="n"/>
       <c r="G105" s="9" t="n"/>
+      <c r="H105" s="9" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -3569,6 +3683,7 @@
       </c>
       <c r="F106" s="5" t="n"/>
       <c r="G106" s="9" t="n"/>
+      <c r="H106" s="9" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -3596,6 +3711,7 @@
       </c>
       <c r="F107" s="5" t="n"/>
       <c r="G107" s="9" t="n"/>
+      <c r="H107" s="9" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -3623,6 +3739,7 @@
       </c>
       <c r="F108" s="5" t="n"/>
       <c r="G108" s="9" t="n"/>
+      <c r="H108" s="9" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3650,6 +3767,7 @@
       </c>
       <c r="F109" s="5" t="n"/>
       <c r="G109" s="9" t="n"/>
+      <c r="H109" s="9" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -3677,6 +3795,7 @@
       </c>
       <c r="F110" s="5" t="n"/>
       <c r="G110" s="9" t="n"/>
+      <c r="H110" s="9" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -3704,6 +3823,7 @@
       </c>
       <c r="F111" s="5" t="n"/>
       <c r="G111" s="9" t="n"/>
+      <c r="H111" s="9" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
@@ -3731,6 +3851,7 @@
       </c>
       <c r="F112" s="5" t="n"/>
       <c r="G112" s="9" t="n"/>
+      <c r="H112" s="9" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -3762,6 +3883,7 @@
           <t>Browni</t>
         </is>
       </c>
+      <c r="H113" s="9" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -3793,6 +3915,7 @@
           <t>Browni</t>
         </is>
       </c>
+      <c r="H114" s="9" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -3824,6 +3947,7 @@
           <t>Unsuz</t>
         </is>
       </c>
+      <c r="H115" s="9" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -3855,6 +3979,7 @@
           <t>Unsuz</t>
         </is>
       </c>
+      <c r="H116" s="9" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -3886,6 +4011,7 @@
           <t>Unsuz</t>
         </is>
       </c>
+      <c r="H117" s="9" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -3917,6 +4043,7 @@
           <t>Unsuz</t>
         </is>
       </c>
+      <c r="H118" s="9" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -3948,6 +4075,7 @@
           <t>Unsuz</t>
         </is>
       </c>
+      <c r="H119" s="9" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -3979,6 +4107,7 @@
           <t>Browni</t>
         </is>
       </c>
+      <c r="H120" s="9" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -4006,6 +4135,7 @@
       </c>
       <c r="F121" s="5" t="n"/>
       <c r="G121" s="9" t="n"/>
+      <c r="H121" s="9" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -4037,6 +4167,7 @@
           <t>Browni</t>
         </is>
       </c>
+      <c r="H122" s="9" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -4064,6 +4195,7 @@
       </c>
       <c r="F123" s="5" t="n"/>
       <c r="G123" s="9" t="n"/>
+      <c r="H123" s="9" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -4095,6 +4227,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H124" s="9" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -4126,6 +4259,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H125" s="9" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4157,6 +4291,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H126" s="9" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -4188,6 +4323,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H127" s="9" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -4219,6 +4355,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H128" s="9" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -4250,6 +4387,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H129" s="9" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
@@ -4281,6 +4419,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H130" s="9" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -4312,6 +4451,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H131" s="9" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
@@ -4343,6 +4483,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H132" s="9" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -4374,6 +4515,7 @@
           <t>Mable</t>
         </is>
       </c>
+      <c r="H133" s="9" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -4405,6 +4547,7 @@
           <t>Bütün Kek</t>
         </is>
       </c>
+      <c r="H134" s="9" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -4436,6 +4579,7 @@
           <t>Bütün Kek</t>
         </is>
       </c>
+      <c r="H135" s="9" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -4467,6 +4611,7 @@
           <t>Bütün Kek</t>
         </is>
       </c>
+      <c r="H136" s="9" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -4498,6 +4643,7 @@
           <t>Bütün Kek</t>
         </is>
       </c>
+      <c r="H137" s="9" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
@@ -4529,6 +4675,7 @@
           <t>Muffin</t>
         </is>
       </c>
+      <c r="H138" s="9" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -4560,6 +4707,7 @@
           <t>Muffin</t>
         </is>
       </c>
+      <c r="H139" s="9" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -4591,6 +4739,7 @@
           <t>Muffin</t>
         </is>
       </c>
+      <c r="H140" s="9" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -4622,6 +4771,7 @@
           <t>Muffin</t>
         </is>
       </c>
+      <c r="H141" s="9" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -4649,6 +4799,7 @@
       </c>
       <c r="F142" s="5" t="n"/>
       <c r="G142" s="9" t="n"/>
+      <c r="H142" s="9" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -4676,6 +4827,7 @@
       </c>
       <c r="F143" s="5" t="n"/>
       <c r="G143" s="9" t="n"/>
+      <c r="H143" s="9" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
@@ -4703,6 +4855,7 @@
       </c>
       <c r="F144" s="5" t="n"/>
       <c r="G144" s="9" t="n"/>
+      <c r="H144" s="9" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -4730,6 +4883,7 @@
       </c>
       <c r="F145" s="5" t="n"/>
       <c r="G145" s="9" t="n"/>
+      <c r="H145" s="9" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
@@ -4757,6 +4911,7 @@
       </c>
       <c r="F146" s="5" t="n"/>
       <c r="G146" s="9" t="n"/>
+      <c r="H146" s="9" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -4784,6 +4939,7 @@
       </c>
       <c r="F147" s="5" t="n"/>
       <c r="G147" s="9" t="n"/>
+      <c r="H147" s="9" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -4811,6 +4967,7 @@
       </c>
       <c r="F148" s="5" t="n"/>
       <c r="G148" s="9" t="n"/>
+      <c r="H148" s="9" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -4838,6 +4995,7 @@
       </c>
       <c r="F149" s="5" t="n"/>
       <c r="G149" s="9" t="n"/>
+      <c r="H149" s="9" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
@@ -4865,6 +5023,7 @@
       </c>
       <c r="F150" s="5" t="n"/>
       <c r="G150" s="9" t="n"/>
+      <c r="H150" s="9" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -4892,6 +5051,7 @@
       </c>
       <c r="F151" s="5" t="n"/>
       <c r="G151" s="9" t="n"/>
+      <c r="H151" s="9" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
@@ -4919,6 +5079,7 @@
       </c>
       <c r="F152" s="5" t="n"/>
       <c r="G152" s="9" t="n"/>
+      <c r="H152" s="9" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -4946,6 +5107,7 @@
       </c>
       <c r="F153" s="5" t="n"/>
       <c r="G153" s="9" t="n"/>
+      <c r="H153" s="9" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -4973,6 +5135,7 @@
       </c>
       <c r="F154" s="5" t="n"/>
       <c r="G154" s="9" t="n"/>
+      <c r="H154" s="9" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -5000,6 +5163,7 @@
       </c>
       <c r="F155" s="5" t="n"/>
       <c r="G155" s="9" t="n"/>
+      <c r="H155" s="9" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -5027,6 +5191,7 @@
       </c>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="9" t="n"/>
+      <c r="H156" s="9" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -5054,6 +5219,7 @@
       </c>
       <c r="F157" s="5" t="n"/>
       <c r="G157" s="9" t="n"/>
+      <c r="H157" s="9" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
@@ -5081,6 +5247,7 @@
       </c>
       <c r="F158" s="5" t="n"/>
       <c r="G158" s="9" t="n"/>
+      <c r="H158" s="9" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -5108,6 +5275,7 @@
       </c>
       <c r="F159" s="5" t="n"/>
       <c r="G159" s="9" t="n"/>
+      <c r="H159" s="9" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
@@ -5135,6 +5303,7 @@
       </c>
       <c r="F160" s="5" t="n"/>
       <c r="G160" s="9" t="n"/>
+      <c r="H160" s="9" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -5162,6 +5331,7 @@
       </c>
       <c r="F161" s="5" t="n"/>
       <c r="G161" s="9" t="n"/>
+      <c r="H161" s="9" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
@@ -5189,6 +5359,7 @@
       </c>
       <c r="F162" s="5" t="n"/>
       <c r="G162" s="9" t="n"/>
+      <c r="H162" s="9" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -5216,6 +5387,7 @@
       </c>
       <c r="F163" s="5" t="n"/>
       <c r="G163" s="9" t="n"/>
+      <c r="H163" s="9" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
@@ -5247,6 +5419,7 @@
           <t>Bar</t>
         </is>
       </c>
+      <c r="H164" s="9" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -5274,6 +5447,7 @@
       </c>
       <c r="F165" s="5" t="n"/>
       <c r="G165" s="9" t="n"/>
+      <c r="H165" s="9" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
@@ -5301,6 +5475,7 @@
       </c>
       <c r="F166" s="5" t="n"/>
       <c r="G166" s="9" t="n"/>
+      <c r="H166" s="9" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -5328,6 +5503,7 @@
       </c>
       <c r="F167" s="5" t="n"/>
       <c r="G167" s="9" t="n"/>
+      <c r="H167" s="9" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -5355,6 +5531,7 @@
       </c>
       <c r="F168" s="5" t="n"/>
       <c r="G168" s="9" t="n"/>
+      <c r="H168" s="9" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -5382,6 +5559,7 @@
       </c>
       <c r="F169" s="5" t="n"/>
       <c r="G169" s="9" t="n"/>
+      <c r="H169" s="9" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -5409,6 +5587,7 @@
       </c>
       <c r="F170" s="5" t="n"/>
       <c r="G170" s="9" t="n"/>
+      <c r="H170" s="9" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -5440,6 +5619,7 @@
           <t>Beze</t>
         </is>
       </c>
+      <c r="H171" s="9" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
@@ -5471,6 +5651,7 @@
           <t>Beze</t>
         </is>
       </c>
+      <c r="H172" s="9" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -5502,6 +5683,7 @@
           <t>Beze</t>
         </is>
       </c>
+      <c r="H173" s="9" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
@@ -5529,6 +5711,7 @@
       </c>
       <c r="F174" s="5" t="n"/>
       <c r="G174" s="9" t="n"/>
+      <c r="H174" s="9" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -5556,6 +5739,7 @@
       </c>
       <c r="F175" s="5" t="n"/>
       <c r="G175" s="9" t="n"/>
+      <c r="H175" s="9" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
@@ -5583,6 +5767,7 @@
       </c>
       <c r="F176" s="5" t="n"/>
       <c r="G176" s="9" t="n"/>
+      <c r="H176" s="9" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -5614,6 +5799,7 @@
           <t>Batonsale</t>
         </is>
       </c>
+      <c r="H177" s="9" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
@@ -5645,6 +5831,7 @@
           <t>Batonsale</t>
         </is>
       </c>
+      <c r="H178" s="9" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -5676,6 +5863,7 @@
           <t>Batonsale</t>
         </is>
       </c>
+      <c r="H179" s="9" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
@@ -5703,6 +5891,7 @@
       </c>
       <c r="F180" s="5" t="n"/>
       <c r="G180" s="9" t="n"/>
+      <c r="H180" s="9" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -5734,6 +5923,7 @@
           <t>Galet</t>
         </is>
       </c>
+      <c r="H181" s="9" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
@@ -5765,6 +5955,7 @@
           <t>Galet</t>
         </is>
       </c>
+      <c r="H182" s="9" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -5796,6 +5987,7 @@
           <t>Galet</t>
         </is>
       </c>
+      <c r="H183" s="9" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
@@ -5827,6 +6019,7 @@
           <t>Kıtır</t>
         </is>
       </c>
+      <c r="H184" s="9" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -5858,6 +6051,7 @@
           <t>Kıtır</t>
         </is>
       </c>
+      <c r="H185" s="9" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
@@ -5889,6 +6083,7 @@
           <t>Kıtır</t>
         </is>
       </c>
+      <c r="H186" s="9" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -5920,6 +6115,7 @@
           <t>Kıtır</t>
         </is>
       </c>
+      <c r="H187" s="9" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
@@ -5951,6 +6147,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H188" s="9" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="inlineStr">
@@ -5982,6 +6179,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H189" s="9" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="inlineStr">
@@ -6013,6 +6211,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H190" s="9" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="inlineStr">
@@ -6044,6 +6243,7 @@
           <t>Cips</t>
         </is>
       </c>
+      <c r="H191" s="9" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -6071,6 +6271,7 @@
       </c>
       <c r="F192" s="5" t="n"/>
       <c r="G192" s="9" t="n"/>
+      <c r="H192" s="9" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="inlineStr">
@@ -6102,6 +6303,7 @@
           <t>Magnolia</t>
         </is>
       </c>
+      <c r="H193" s="9" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="inlineStr">
@@ -6133,6 +6335,7 @@
           <t>Magnolia</t>
         </is>
       </c>
+      <c r="H194" s="9" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="inlineStr">
@@ -6164,6 +6367,7 @@
           <t>Magnolia</t>
         </is>
       </c>
+      <c r="H195" s="9" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="inlineStr">
@@ -6195,6 +6399,7 @@
           <t>Magnolia</t>
         </is>
       </c>
+      <c r="H196" s="9" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="inlineStr">
@@ -6222,6 +6427,7 @@
       </c>
       <c r="F197" s="5" t="n"/>
       <c r="G197" s="9" t="n"/>
+      <c r="H197" s="9" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="inlineStr">
@@ -6249,6 +6455,7 @@
       </c>
       <c r="F198" s="5" t="n"/>
       <c r="G198" s="9" t="n"/>
+      <c r="H198" s="9" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="inlineStr">
@@ -6276,6 +6483,7 @@
       </c>
       <c r="F199" s="5" t="n"/>
       <c r="G199" s="9" t="n"/>
+      <c r="H199" s="9" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="inlineStr">
@@ -6303,6 +6511,7 @@
       </c>
       <c r="F200" s="5" t="n"/>
       <c r="G200" s="9" t="n"/>
+      <c r="H200" s="9" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="inlineStr">
@@ -6330,6 +6539,7 @@
       </c>
       <c r="F201" s="5" t="n"/>
       <c r="G201" s="9" t="n"/>
+      <c r="H201" s="9" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="3" t="inlineStr">
@@ -6357,6 +6567,7 @@
       </c>
       <c r="F202" s="5" t="n"/>
       <c r="G202" s="9" t="n"/>
+      <c r="H202" s="9" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="3" t="inlineStr">
@@ -6384,6 +6595,7 @@
       </c>
       <c r="F203" s="5" t="n"/>
       <c r="G203" s="9" t="n"/>
+      <c r="H203" s="9" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="3" t="inlineStr">
@@ -6411,6 +6623,7 @@
       </c>
       <c r="F204" s="5" t="n"/>
       <c r="G204" s="9" t="n"/>
+      <c r="H204" s="9" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="3" t="inlineStr">
@@ -6438,6 +6651,7 @@
       </c>
       <c r="F205" s="5" t="n"/>
       <c r="G205" s="9" t="n"/>
+      <c r="H205" s="9" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="3" t="inlineStr">
@@ -6465,6 +6679,7 @@
       </c>
       <c r="F206" s="5" t="n"/>
       <c r="G206" s="9" t="n"/>
+      <c r="H206" s="9" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -6492,6 +6707,7 @@
       </c>
       <c r="F207" s="5" t="n"/>
       <c r="G207" s="9" t="n"/>
+      <c r="H207" s="9" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="3" t="inlineStr">
@@ -6519,6 +6735,7 @@
       </c>
       <c r="F208" s="5" t="n"/>
       <c r="G208" s="9" t="n"/>
+      <c r="H208" s="9" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="8" t="inlineStr">
@@ -6550,6 +6767,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H209" s="9" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="3" t="inlineStr">
@@ -6581,6 +6799,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H210" s="9" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="3" t="inlineStr">
@@ -6612,6 +6831,7 @@
           <t>Ekler</t>
         </is>
       </c>
+      <c r="H211" s="9" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="3" t="inlineStr">
@@ -6643,6 +6863,7 @@
           <t>Petifür &amp; Rulo</t>
         </is>
       </c>
+      <c r="H212" s="9" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="3" t="inlineStr">
@@ -6674,6 +6895,7 @@
           <t>Petifür &amp; Rulo</t>
         </is>
       </c>
+      <c r="H213" s="9" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="3" t="inlineStr">
@@ -6705,6 +6927,7 @@
           <t>Petifür &amp; Rulo</t>
         </is>
       </c>
+      <c r="H214" s="9" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="3" t="inlineStr">
@@ -6732,6 +6955,7 @@
       </c>
       <c r="F215" s="5" t="n"/>
       <c r="G215" s="9" t="n"/>
+      <c r="H215" s="9" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="3" t="inlineStr">
@@ -6763,6 +6987,7 @@
           <t>Petifür &amp; Rulo</t>
         </is>
       </c>
+      <c r="H216" s="9" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="3" t="inlineStr">
@@ -6794,6 +7019,7 @@
           <t>Petifür &amp; Rulo</t>
         </is>
       </c>
+      <c r="H217" s="9" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="3" t="inlineStr">
@@ -6825,6 +7051,7 @@
           <t>Şu Topu</t>
         </is>
       </c>
+      <c r="H218" s="9" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="3" t="inlineStr">
@@ -6856,6 +7083,7 @@
           <t>Şu Topu</t>
         </is>
       </c>
+      <c r="H219" s="9" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -6883,6 +7111,7 @@
       </c>
       <c r="F220" s="5" t="n"/>
       <c r="G220" s="9" t="n"/>
+      <c r="H220" s="9" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="3" t="inlineStr">
@@ -6910,6 +7139,7 @@
       </c>
       <c r="F221" s="5" t="n"/>
       <c r="G221" s="9" t="n"/>
+      <c r="H221" s="9" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="3" t="inlineStr">
@@ -6937,6 +7167,7 @@
       </c>
       <c r="F222" s="5" t="n"/>
       <c r="G222" s="9" t="n"/>
+      <c r="H222" s="9" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="3" t="inlineStr">
@@ -6968,6 +7199,7 @@
           <t>Trileçe</t>
         </is>
       </c>
+      <c r="H223" s="9" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="3" t="inlineStr">
@@ -6999,6 +7231,7 @@
           <t>Trileçe</t>
         </is>
       </c>
+      <c r="H224" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7012,7 +7245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -7094,7 +7327,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>birim / boylu : Sadece bilgi amaçlı, dokunmayın.</t>
+          <t>birim  : Ürün adının yanında parantezde yazılır. BOŞ bırakırsanız hiç yazılmaz.</t>
         </is>
       </c>
     </row>
@@ -7119,6 +7352,41 @@
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>tablodaki görünme sırasına göre belirlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>ALT GRUP   : Bölüm içindeki alt grup. Grup değiştiğinde araya ince bir</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             boş satır konur. Boş bırakılırsa ayırıcı konmaz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>GÖRÜNEN AD : Raporda bu ad yazılır. Boş bırakılırsa ÜRÜN sütunundaki ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             kullanılır. ÜRÜN sütununu değiştirmeden adı değiştirmek için.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>boylu      : Sadece bilgi amaçlı, dokunmayın.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ayçekirdekli Galeta, Kornet Dereotlu, Dereotlu Sufle birimi: kg
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -4924,7 +4924,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F146" s="5" t="n"/>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>tp</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="F147" s="5" t="n"/>
@@ -5238,7 +5238,11 @@
       <c r="D156" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E156" s="5" t="n"/>
+      <c r="E156" s="5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
       <c r="F156" s="5" t="n"/>
       <c r="G156" s="9" t="n"/>
       <c r="H156" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Rapor düzenindeki sıralama değişikliklerini uygula; 2 kurabiyeyi çıkar
</commit_message>
<xml_diff>
--- a/rapor-duzeni.xlsx
+++ b/rapor-duzeni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/serkansalihoglu/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D90DA66-C324-864B-8D86-63FCA0B5BC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B855EF-4572-3B42-98B5-A932D976EA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16600" yWindow="860" windowWidth="21060" windowHeight="17040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="311">
   <si>
     <t>SAYFA</t>
   </si>
@@ -417,12 +417,6 @@
   </si>
   <si>
     <t>Vişneli Bar</t>
-  </si>
-  <si>
-    <t>Karamelli Yıldız Kurabiye</t>
-  </si>
-  <si>
-    <t>Şekilli Kurabiye</t>
   </si>
   <si>
     <t>Elmalı Kurabiye</t>
@@ -1066,7 +1060,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1082,6 +1076,8 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1384,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H220"/>
+  <dimension ref="A1:H218"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3440,43 +3436,47 @@
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A98" s="3" t="s">
+      <c r="A98" s="11" t="s">
         <v>101</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>102</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="D98" s="4">
         <v>26</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
-      <c r="G98" s="9"/>
+      <c r="G98" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="H98" s="3" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A99" s="3" t="s">
+      <c r="A99" s="12" t="s">
         <v>101</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>102</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="D99" s="4">
         <v>27</v>
       </c>
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
-      <c r="G99" s="9"/>
+      <c r="G99" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="H99" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
@@ -3487,7 +3487,7 @@
         <v>102</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D100" s="4">
         <v>28</v>
@@ -3496,7 +3496,7 @@
       <c r="F100" s="5"/>
       <c r="G100" s="9"/>
       <c r="H100" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
@@ -3507,7 +3507,7 @@
         <v>102</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D101" s="4">
         <v>29</v>
@@ -3516,7 +3516,7 @@
       <c r="F101" s="5"/>
       <c r="G101" s="9"/>
       <c r="H101" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
@@ -3527,7 +3527,7 @@
         <v>102</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D102" s="4">
         <v>30</v>
@@ -3536,7 +3536,7 @@
       <c r="F102" s="5"/>
       <c r="G102" s="9"/>
       <c r="H102" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
@@ -3547,7 +3547,7 @@
         <v>102</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D103" s="4">
         <v>31</v>
@@ -3556,7 +3556,7 @@
       <c r="F103" s="5"/>
       <c r="G103" s="9"/>
       <c r="H103" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
@@ -3567,7 +3567,7 @@
         <v>102</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D104" s="4">
         <v>32</v>
@@ -3576,7 +3576,7 @@
       <c r="F104" s="5"/>
       <c r="G104" s="9"/>
       <c r="H104" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
@@ -3587,7 +3587,7 @@
         <v>102</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D105" s="4">
         <v>33</v>
@@ -3596,7 +3596,7 @@
       <c r="F105" s="5"/>
       <c r="G105" s="9"/>
       <c r="H105" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
@@ -3607,7 +3607,7 @@
         <v>102</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D106" s="4">
         <v>34</v>
@@ -3616,7 +3616,7 @@
       <c r="F106" s="5"/>
       <c r="G106" s="9"/>
       <c r="H106" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.2">
@@ -3627,7 +3627,7 @@
         <v>102</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D107" s="4">
         <v>35</v>
@@ -3636,7 +3636,7 @@
       <c r="F107" s="5"/>
       <c r="G107" s="9"/>
       <c r="H107" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
@@ -3647,7 +3647,7 @@
         <v>102</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D108" s="4">
         <v>36</v>
@@ -3656,7 +3656,7 @@
       <c r="F108" s="5"/>
       <c r="G108" s="9"/>
       <c r="H108" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
@@ -3667,7 +3667,7 @@
         <v>102</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D109" s="4">
         <v>37</v>
@@ -3676,7 +3676,7 @@
       <c r="F109" s="5"/>
       <c r="G109" s="9"/>
       <c r="H109" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.2">
@@ -3687,7 +3687,7 @@
         <v>102</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D110" s="4">
         <v>38</v>
@@ -3696,7 +3696,7 @@
       <c r="F110" s="5"/>
       <c r="G110" s="9"/>
       <c r="H110" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
@@ -3707,7 +3707,7 @@
         <v>102</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D111" s="4">
         <v>39</v>
@@ -3716,7 +3716,7 @@
       <c r="F111" s="5"/>
       <c r="G111" s="9"/>
       <c r="H111" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.2">
@@ -3727,7 +3727,7 @@
         <v>102</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D112" s="4">
         <v>40</v>
@@ -3736,7 +3736,7 @@
       <c r="F112" s="5"/>
       <c r="G112" s="9"/>
       <c r="H112" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
@@ -3744,10 +3744,10 @@
         <v>101</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D113" s="4">
         <v>1</v>
@@ -3755,10 +3755,10 @@
       <c r="E113" s="5"/>
       <c r="F113" s="5"/>
       <c r="G113" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="H113" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="H113" s="3" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
@@ -3766,7 +3766,7 @@
         <v>101</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>150</v>
@@ -3777,7 +3777,7 @@
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
       <c r="G114" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>150</v>
@@ -3788,7 +3788,7 @@
         <v>101</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>151</v>
@@ -3799,7 +3799,7 @@
       <c r="E115" s="5"/>
       <c r="F115" s="5"/>
       <c r="G115" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>151</v>
@@ -3810,7 +3810,7 @@
         <v>101</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>152</v>
@@ -3821,7 +3821,7 @@
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
       <c r="G116" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>152</v>
@@ -3832,7 +3832,7 @@
         <v>101</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>153</v>
@@ -3843,7 +3843,7 @@
       <c r="E117" s="5"/>
       <c r="F117" s="5"/>
       <c r="G117" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>153</v>
@@ -3854,7 +3854,7 @@
         <v>101</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>154</v>
@@ -3876,7 +3876,7 @@
         <v>101</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>155</v>
@@ -3886,9 +3886,7 @@
       </c>
       <c r="E119" s="5"/>
       <c r="F119" s="5"/>
-      <c r="G119" s="9" t="s">
-        <v>147</v>
-      </c>
+      <c r="G119" s="9"/>
       <c r="H119" s="3" t="s">
         <v>155</v>
       </c>
@@ -3898,7 +3896,7 @@
         <v>101</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>156</v>
@@ -3909,7 +3907,7 @@
       <c r="E120" s="5"/>
       <c r="F120" s="5"/>
       <c r="G120" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H120" s="3" t="s">
         <v>156</v>
@@ -3920,7 +3918,7 @@
         <v>101</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>157</v>
@@ -3940,7 +3938,7 @@
         <v>101</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>158</v>
@@ -3951,7 +3949,7 @@
       <c r="E122" s="5"/>
       <c r="F122" s="5"/>
       <c r="G122" s="9" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>158</v>
@@ -3962,41 +3960,43 @@
         <v>101</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D123" s="4">
         <v>11</v>
       </c>
       <c r="E123" s="5"/>
       <c r="F123" s="5"/>
-      <c r="G123" s="9"/>
+      <c r="G123" s="9" t="s">
+        <v>159</v>
+      </c>
       <c r="H123" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A124" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B124" s="3" t="s">
-        <v>147</v>
+      <c r="A124" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D124" s="4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
       <c r="G124" s="9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H124" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.2">
@@ -4004,43 +4004,43 @@
         <v>101</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D125" s="4">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E125" s="5"/>
       <c r="F125" s="5"/>
       <c r="G125" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H125" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A126" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B126" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="H125" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A126" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="C126" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D126" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E126" s="5"/>
       <c r="F126" s="5"/>
       <c r="G126" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="H126" s="3" t="s">
         <v>165</v>
-      </c>
-      <c r="H126" s="3" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.2">
@@ -4048,18 +4048,18 @@
         <v>101</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>166</v>
       </c>
       <c r="D127" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E127" s="5"/>
       <c r="F127" s="5"/>
       <c r="G127" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H127" s="3" t="s">
         <v>166</v>
@@ -4070,18 +4070,18 @@
         <v>101</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>167</v>
       </c>
       <c r="D128" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E128" s="5"/>
       <c r="F128" s="5"/>
       <c r="G128" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H128" s="3" t="s">
         <v>167</v>
@@ -4092,18 +4092,18 @@
         <v>101</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>168</v>
       </c>
       <c r="D129" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
       <c r="G129" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H129" s="3" t="s">
         <v>168</v>
@@ -4114,18 +4114,18 @@
         <v>101</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>169</v>
       </c>
       <c r="D130" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E130" s="5"/>
       <c r="F130" s="5"/>
       <c r="G130" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H130" s="3" t="s">
         <v>169</v>
@@ -4136,18 +4136,18 @@
         <v>101</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>170</v>
       </c>
       <c r="D131" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
       <c r="G131" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H131" s="3" t="s">
         <v>170</v>
@@ -4158,21 +4158,21 @@
         <v>101</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>171</v>
       </c>
       <c r="D132" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
       <c r="G132" s="9" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.2">
@@ -4180,21 +4180,21 @@
         <v>101</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D133" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5"/>
       <c r="G133" s="9" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.2">
@@ -4202,21 +4202,21 @@
         <v>101</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D134" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E134" s="5"/>
       <c r="F134" s="5"/>
       <c r="G134" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.2">
@@ -4224,21 +4224,21 @@
         <v>101</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D135" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
       <c r="G135" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.2">
@@ -4246,21 +4246,21 @@
         <v>101</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D136" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E136" s="5"/>
       <c r="F136" s="5"/>
       <c r="G136" s="9" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.2">
@@ -4268,21 +4268,21 @@
         <v>101</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D137" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="9" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.2">
@@ -4290,21 +4290,21 @@
         <v>101</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D138" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="H138" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="H138" s="3" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.2">
@@ -4312,104 +4312,104 @@
         <v>101</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C139" s="3" t="s">
         <v>184</v>
       </c>
       <c r="D139" s="4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
       <c r="G139" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H139" s="3" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A140" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B140" s="3" t="s">
-        <v>163</v>
+      <c r="A140" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>186</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D140" s="4">
-        <v>15</v>
-      </c>
-      <c r="E140" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>188</v>
+      </c>
       <c r="F140" s="5"/>
-      <c r="G140" s="9" t="s">
-        <v>183</v>
-      </c>
+      <c r="G140" s="9"/>
       <c r="H140" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
-        <v>101</v>
+        <v>185</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="C141" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D141" s="4">
+        <v>2</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F141" s="5"/>
+      <c r="G141" s="9"/>
+      <c r="H141" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A142" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B142" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D141" s="4">
-        <v>16</v>
-      </c>
-      <c r="E141" s="5"/>
-      <c r="F141" s="5"/>
-      <c r="G141" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="H141" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A142" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B142" s="2" t="s">
+      <c r="C142" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D142" s="4">
+        <v>3</v>
+      </c>
+      <c r="E142" s="5" t="s">
         <v>188</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="D142" s="4">
-        <v>1</v>
-      </c>
-      <c r="E142" s="5" t="s">
-        <v>190</v>
       </c>
       <c r="F142" s="5"/>
       <c r="G142" s="9"/>
       <c r="H142" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>191</v>
       </c>
       <c r="D143" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E143" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F143" s="5"/>
       <c r="G143" s="9"/>
@@ -4419,19 +4419,19 @@
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A144" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>192</v>
       </c>
       <c r="D144" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F144" s="5"/>
       <c r="G144" s="9"/>
@@ -4441,63 +4441,63 @@
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C145" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D145" s="4">
+        <v>6</v>
+      </c>
+      <c r="E145" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="D145" s="4">
-        <v>4</v>
-      </c>
-      <c r="E145" s="5" t="s">
-        <v>190</v>
       </c>
       <c r="F145" s="5"/>
       <c r="G145" s="9"/>
       <c r="H145" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A146" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B146" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D146" s="4">
+        <v>7</v>
+      </c>
+      <c r="E146" s="5" t="s">
         <v>188</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="D146" s="4">
-        <v>5</v>
-      </c>
-      <c r="E146" s="5" t="s">
-        <v>195</v>
       </c>
       <c r="F146" s="5"/>
       <c r="G146" s="9"/>
       <c r="H146" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C147" s="3" t="s">
         <v>196</v>
       </c>
       <c r="D147" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E147" s="5" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F147" s="5"/>
       <c r="G147" s="9"/>
@@ -4507,19 +4507,19 @@
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C148" s="3" t="s">
         <v>197</v>
       </c>
       <c r="D148" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F148" s="5"/>
       <c r="G148" s="9"/>
@@ -4529,19 +4529,19 @@
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A149" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C149" s="3" t="s">
         <v>198</v>
       </c>
       <c r="D149" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E149" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F149" s="5"/>
       <c r="G149" s="9"/>
@@ -4551,19 +4551,19 @@
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A150" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C150" s="3" t="s">
         <v>199</v>
       </c>
       <c r="D150" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E150" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F150" s="5"/>
       <c r="G150" s="9"/>
@@ -4573,19 +4573,19 @@
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A151" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C151" s="3" t="s">
         <v>200</v>
       </c>
       <c r="D151" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F151" s="5"/>
       <c r="G151" s="9"/>
@@ -4595,19 +4595,19 @@
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A152" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C152" s="3" t="s">
         <v>201</v>
       </c>
       <c r="D152" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F152" s="5"/>
       <c r="G152" s="9"/>
@@ -4616,63 +4616,63 @@
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A153" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B153" s="3" t="s">
-        <v>188</v>
+      <c r="A153" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D153" s="4">
-        <v>12</v>
-      </c>
-      <c r="E153" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E153" s="5"/>
       <c r="F153" s="5"/>
       <c r="G153" s="9"/>
       <c r="H153" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A154" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D154" s="4">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F154" s="5"/>
       <c r="G154" s="9"/>
       <c r="H154" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A155" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B155" s="2" t="s">
-        <v>204</v>
+      <c r="A155" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>202</v>
       </c>
       <c r="C155" s="3" t="s">
         <v>205</v>
       </c>
       <c r="D155" s="4">
-        <v>1</v>
-      </c>
-      <c r="E155" s="5"/>
+        <v>3</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>188</v>
+      </c>
       <c r="F155" s="5"/>
       <c r="G155" s="9"/>
       <c r="H155" s="3" t="s">
@@ -4681,19 +4681,19 @@
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A156" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C156" s="3" t="s">
         <v>206</v>
       </c>
       <c r="D156" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F156" s="5"/>
       <c r="G156" s="9"/>
@@ -4703,19 +4703,19 @@
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C157" s="3" t="s">
         <v>207</v>
       </c>
       <c r="D157" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E157" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F157" s="5"/>
       <c r="G157" s="9"/>
@@ -4725,19 +4725,19 @@
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A158" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C158" s="3" t="s">
         <v>208</v>
       </c>
       <c r="D158" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F158" s="5"/>
       <c r="G158" s="9"/>
@@ -4747,19 +4747,19 @@
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C159" s="3" t="s">
         <v>209</v>
       </c>
       <c r="D159" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F159" s="5"/>
       <c r="G159" s="9"/>
@@ -4769,19 +4769,19 @@
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C160" s="3" t="s">
         <v>210</v>
       </c>
       <c r="D160" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F160" s="5"/>
       <c r="G160" s="9"/>
@@ -4791,20 +4791,18 @@
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C161" s="3" t="s">
         <v>211</v>
       </c>
       <c r="D161" s="4">
-        <v>7</v>
-      </c>
-      <c r="E161" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="E161" s="5"/>
       <c r="F161" s="5"/>
       <c r="G161" s="9"/>
       <c r="H161" s="3" t="s">
@@ -4813,38 +4811,38 @@
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C162" s="3" t="s">
         <v>212</v>
       </c>
       <c r="D162" s="4">
-        <v>8</v>
-      </c>
-      <c r="E162" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E162" s="5"/>
       <c r="F162" s="5"/>
-      <c r="G162" s="9"/>
+      <c r="G162" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="H162" s="3" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A163" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C163" s="3" t="s">
         <v>213</v>
       </c>
       <c r="D163" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E163" s="5"/>
       <c r="F163" s="5"/>
@@ -4855,38 +4853,36 @@
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A164" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C164" s="3" t="s">
         <v>214</v>
       </c>
       <c r="D164" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E164" s="5"/>
       <c r="F164" s="5"/>
-      <c r="G164" s="9" t="s">
-        <v>129</v>
-      </c>
+      <c r="G164" s="9"/>
       <c r="H164" s="3" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A165" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C165" s="3" t="s">
         <v>215</v>
       </c>
       <c r="D165" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E165" s="5"/>
       <c r="F165" s="5"/>
@@ -4896,57 +4892,57 @@
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A166" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B166" s="3" t="s">
-        <v>204</v>
+      <c r="A166" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D166" s="4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E166" s="5"/>
       <c r="F166" s="5"/>
       <c r="G166" s="9"/>
       <c r="H166" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D167" s="4">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E167" s="5"/>
       <c r="F167" s="5"/>
       <c r="G167" s="9"/>
       <c r="H167" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A168" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B168" s="2" t="s">
-        <v>218</v>
+      <c r="A168" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>216</v>
       </c>
       <c r="C168" s="3" t="s">
         <v>219</v>
       </c>
       <c r="D168" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
@@ -4957,122 +4953,122 @@
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C169" s="3" t="s">
         <v>220</v>
       </c>
       <c r="D169" s="4">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E169" s="5"/>
       <c r="F169" s="5"/>
-      <c r="G169" s="9"/>
+      <c r="G169" s="9" t="s">
+        <v>221</v>
+      </c>
       <c r="H169" s="3" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D170" s="4">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E170" s="5"/>
       <c r="F170" s="5"/>
-      <c r="G170" s="9"/>
+      <c r="G170" s="9" t="s">
+        <v>221</v>
+      </c>
       <c r="H170" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D171" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E171" s="5"/>
       <c r="F171" s="5"/>
       <c r="G171" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="H171" s="3" t="s">
         <v>223</v>
-      </c>
-      <c r="H171" s="3" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A172" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C172" s="3" t="s">
         <v>224</v>
       </c>
       <c r="D172" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E172" s="5"/>
       <c r="F172" s="5"/>
-      <c r="G172" s="9" t="s">
-        <v>223</v>
-      </c>
+      <c r="G172" s="9"/>
       <c r="H172" s="3" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C173" s="3" t="s">
         <v>225</v>
       </c>
       <c r="D173" s="4">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E173" s="5"/>
       <c r="F173" s="5"/>
-      <c r="G173" s="9" t="s">
-        <v>223</v>
-      </c>
+      <c r="G173" s="9"/>
       <c r="H173" s="3" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A174" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C174" s="3" t="s">
         <v>226</v>
       </c>
       <c r="D174" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E174" s="5"/>
       <c r="F174" s="5"/>
@@ -5082,112 +5078,118 @@
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A175" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B175" s="3" t="s">
-        <v>218</v>
+      <c r="A175" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B175" s="2" t="s">
+        <v>227</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D175" s="4">
-        <v>5</v>
-      </c>
-      <c r="E175" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="E175" s="5" t="s">
+        <v>188</v>
+      </c>
       <c r="F175" s="5"/>
-      <c r="G175" s="9"/>
+      <c r="G175" s="9" t="s">
+        <v>229</v>
+      </c>
       <c r="H175" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D176" s="4">
-        <v>6</v>
-      </c>
-      <c r="E176" s="5"/>
+        <v>2</v>
+      </c>
+      <c r="E176" s="5" t="s">
+        <v>188</v>
+      </c>
       <c r="F176" s="5"/>
-      <c r="G176" s="9"/>
+      <c r="G176" s="9" t="s">
+        <v>229</v>
+      </c>
       <c r="H176" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A177" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B177" s="2" t="s">
-        <v>229</v>
+      <c r="A177" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>227</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D177" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E177" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F177" s="5"/>
       <c r="G177" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="H177" s="3" t="s">
         <v>231</v>
-      </c>
-      <c r="H177" s="3" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C178" s="3" t="s">
         <v>232</v>
       </c>
       <c r="D178" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E178" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F178" s="5"/>
-      <c r="G178" s="9" t="s">
-        <v>231</v>
-      </c>
+      <c r="G178" s="9"/>
       <c r="H178" s="3" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A179" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B179" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C179" s="3" t="s">
         <v>233</v>
       </c>
       <c r="D179" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E179" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F179" s="5"/>
       <c r="G179" s="9" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="H179" s="3" t="s">
         <v>233</v>
@@ -5195,69 +5197,71 @@
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C180" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D180" s="4">
+        <v>6</v>
+      </c>
+      <c r="E180" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F180" s="5"/>
+      <c r="G180" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="D180" s="4">
-        <v>4</v>
-      </c>
-      <c r="E180" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="F180" s="5"/>
-      <c r="G180" s="9"/>
       <c r="H180" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A181" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D181" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F181" s="5"/>
       <c r="G181" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="H181" s="3" t="s">
         <v>236</v>
-      </c>
-      <c r="H181" s="3" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A182" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C182" s="3" t="s">
         <v>237</v>
       </c>
       <c r="D182" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E182" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F182" s="5"/>
       <c r="G182" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H182" s="3" t="s">
         <v>237</v>
@@ -5265,71 +5269,71 @@
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A183" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D183" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E183" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F183" s="5"/>
       <c r="G183" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H183" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D184" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E184" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F184" s="5"/>
       <c r="G184" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="H184" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="H184" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A185" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C185" s="3" t="s">
         <v>241</v>
       </c>
       <c r="D185" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E185" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F185" s="5"/>
       <c r="G185" s="9" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H185" s="3" t="s">
         <v>241</v>
@@ -5337,23 +5341,23 @@
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A186" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C186" s="3" t="s">
         <v>242</v>
       </c>
       <c r="D186" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E186" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F186" s="5"/>
       <c r="G186" s="9" t="s">
-        <v>240</v>
+        <v>159</v>
       </c>
       <c r="H186" s="3" t="s">
         <v>242</v>
@@ -5361,23 +5365,23 @@
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A187" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C187" s="3" t="s">
         <v>243</v>
       </c>
       <c r="D187" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E187" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F187" s="5"/>
       <c r="G187" s="9" t="s">
-        <v>240</v>
+        <v>159</v>
       </c>
       <c r="H187" s="3" t="s">
         <v>243</v>
@@ -5385,23 +5389,23 @@
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A188" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C188" s="3" t="s">
         <v>244</v>
       </c>
       <c r="D188" s="4">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E188" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F188" s="5"/>
       <c r="G188" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H188" s="3" t="s">
         <v>244</v>
@@ -5409,135 +5413,131 @@
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A189" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C189" s="3" t="s">
         <v>245</v>
       </c>
       <c r="D189" s="4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E189" s="5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F189" s="5"/>
       <c r="G189" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H189" s="3" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A190" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B190" s="3" t="s">
-        <v>229</v>
+      <c r="A190" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D190" s="4">
-        <v>14</v>
-      </c>
-      <c r="E190" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E190" s="5"/>
       <c r="F190" s="5"/>
-      <c r="G190" s="9" t="s">
-        <v>161</v>
-      </c>
+      <c r="G190" s="9"/>
       <c r="H190" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A191" s="3" t="s">
-        <v>187</v>
+        <v>246</v>
       </c>
       <c r="B191" s="3" t="s">
-        <v>229</v>
+        <v>246</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D191" s="4">
-        <v>15</v>
-      </c>
-      <c r="E191" s="5" t="s">
-        <v>190</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E191" s="5"/>
       <c r="F191" s="5"/>
       <c r="G191" s="9" t="s">
-        <v>161</v>
+        <v>249</v>
       </c>
       <c r="H191" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A192" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B192" s="2" t="s">
-        <v>248</v>
+      <c r="A192" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>246</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D192" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E192" s="5"/>
       <c r="F192" s="5"/>
-      <c r="G192" s="9"/>
+      <c r="G192" s="9" t="s">
+        <v>249</v>
+      </c>
       <c r="H192" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D193" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E193" s="5"/>
       <c r="F193" s="5"/>
       <c r="G193" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="H193" s="3" t="s">
         <v>251</v>
-      </c>
-      <c r="H193" s="3" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A194" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C194" s="3" t="s">
         <v>252</v>
       </c>
       <c r="D194" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E194" s="5"/>
       <c r="F194" s="5"/>
       <c r="G194" s="9" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H194" s="3" t="s">
         <v>252</v>
@@ -5545,60 +5545,56 @@
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A195" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C195" s="3" t="s">
         <v>253</v>
       </c>
       <c r="D195" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E195" s="5"/>
       <c r="F195" s="5"/>
-      <c r="G195" s="9" t="s">
-        <v>251</v>
-      </c>
+      <c r="G195" s="9"/>
       <c r="H195" s="3" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A196" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C196" s="3" t="s">
         <v>254</v>
       </c>
       <c r="D196" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E196" s="5"/>
       <c r="F196" s="5"/>
-      <c r="G196" s="9" t="s">
-        <v>251</v>
-      </c>
+      <c r="G196" s="9"/>
       <c r="H196" s="3" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C197" s="3" t="s">
         <v>255</v>
       </c>
       <c r="D197" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E197" s="5"/>
       <c r="F197" s="5"/>
@@ -5609,16 +5605,16 @@
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B198" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C198" s="3" t="s">
         <v>256</v>
       </c>
       <c r="D198" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E198" s="5"/>
       <c r="F198" s="5"/>
@@ -5629,16 +5625,16 @@
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A199" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C199" s="3" t="s">
         <v>257</v>
       </c>
       <c r="D199" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E199" s="5"/>
       <c r="F199" s="5"/>
@@ -5649,16 +5645,16 @@
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C200" s="3" t="s">
         <v>258</v>
       </c>
       <c r="D200" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
@@ -5669,16 +5665,16 @@
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C201" s="3" t="s">
         <v>259</v>
       </c>
       <c r="D201" s="4">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E201" s="5"/>
       <c r="F201" s="5"/>
@@ -5689,76 +5685,80 @@
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A202" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C202" s="3" t="s">
         <v>260</v>
       </c>
       <c r="D202" s="4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E202" s="5"/>
       <c r="F202" s="5"/>
       <c r="G202" s="9"/>
       <c r="H202" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A203" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B203" s="3" t="s">
-        <v>248</v>
+      <c r="A203" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B203" s="8" t="s">
+        <v>262</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D203" s="4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E203" s="5"/>
       <c r="F203" s="5"/>
-      <c r="G203" s="9"/>
+      <c r="G203" s="9" t="s">
+        <v>38</v>
+      </c>
       <c r="H203" s="3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D204" s="4">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E204" s="5"/>
       <c r="F204" s="5"/>
-      <c r="G204" s="9"/>
+      <c r="G204" s="9" t="s">
+        <v>38</v>
+      </c>
       <c r="H204" s="3" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A205" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="B205" s="8" t="s">
-        <v>264</v>
+      <c r="A205" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B205" s="3" t="s">
+        <v>262</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D205" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E205" s="5"/>
       <c r="F205" s="5"/>
@@ -5766,156 +5766,156 @@
         <v>38</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A206" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B206" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D206" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E206" s="5"/>
       <c r="F206" s="5"/>
       <c r="G206" s="9" t="s">
-        <v>38</v>
+        <v>270</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A207" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D207" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E207" s="5"/>
       <c r="F207" s="5"/>
       <c r="G207" s="9" t="s">
-        <v>38</v>
+        <v>270</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A208" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D208" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E208" s="5"/>
       <c r="F208" s="5"/>
       <c r="G208" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A209" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="D209" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E209" s="5"/>
       <c r="F209" s="5"/>
-      <c r="G209" s="9" t="s">
-        <v>272</v>
-      </c>
+      <c r="G209" s="9"/>
       <c r="H209" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D210" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E210" s="5"/>
       <c r="F210" s="5"/>
       <c r="G210" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D211" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E211" s="5"/>
       <c r="F211" s="5"/>
-      <c r="G211" s="9"/>
+      <c r="G211" s="9" t="s">
+        <v>270</v>
+      </c>
       <c r="H211" s="3" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C212" s="3" t="s">
         <v>280</v>
       </c>
       <c r="D212" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E212" s="5"/>
       <c r="F212" s="5"/>
       <c r="G212" s="9" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="H212" s="3" t="s">
         <v>280</v>
@@ -5923,82 +5923,78 @@
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D213" s="4">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E213" s="5"/>
       <c r="F213" s="5"/>
       <c r="G213" s="9" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="214" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A214" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B214" s="3" t="s">
-        <v>264</v>
+      <c r="A214" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>283</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D214" s="4">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E214" s="5"/>
       <c r="F214" s="5"/>
-      <c r="G214" s="9" t="s">
-        <v>283</v>
-      </c>
+      <c r="G214" s="9"/>
       <c r="H214" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>264</v>
+        <v>283</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D215" s="4">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E215" s="5"/>
       <c r="F215" s="5"/>
-      <c r="G215" s="9" t="s">
+      <c r="G215" s="9"/>
+      <c r="H215" s="3" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A216" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B216" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="H215" s="3" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A216" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B216" s="2" t="s">
-        <v>285</v>
       </c>
       <c r="C216" s="3" t="s">
         <v>286</v>
       </c>
       <c r="D216" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E216" s="5"/>
       <c r="F216" s="5"/>
@@ -6009,86 +6005,46 @@
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>285</v>
+        <v>246</v>
       </c>
       <c r="C217" s="3" t="s">
         <v>287</v>
       </c>
       <c r="D217" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E217" s="5"/>
       <c r="F217" s="5"/>
-      <c r="G217" s="9"/>
+      <c r="G217" s="9" t="s">
+        <v>288</v>
+      </c>
       <c r="H217" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A218" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>285</v>
+        <v>246</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D218" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E218" s="5"/>
       <c r="F218" s="5"/>
-      <c r="G218" s="9"/>
+      <c r="G218" s="9" t="s">
+        <v>288</v>
+      </c>
       <c r="H218" s="3" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A219" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B219" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="C219" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D219" s="4">
-        <v>1</v>
-      </c>
-      <c r="E219" s="5"/>
-      <c r="F219" s="5"/>
-      <c r="G219" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="H219" s="3" t="s">
         <v>291</v>
-      </c>
-    </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A220" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B220" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D220" s="4">
-        <v>2</v>
-      </c>
-      <c r="E220" s="5"/>
-      <c r="F220" s="5"/>
-      <c r="G220" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="H220" s="3" t="s">
-        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -6107,12 +6063,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
@@ -6120,47 +6076,47 @@
     </row>
     <row r="4" spans="1:1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
@@ -6168,42 +6124,42 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>